<commit_message>
Updated Selenium framework and added BDD project
</commit_message>
<xml_diff>
--- a/Selenium_Framework/data/product.xlsx
+++ b/Selenium_Framework/data/product.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aziz Shaik\Desktop\Myntra_Capstone_Project\Selenium_Framework\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19D15A33-642E-4EF3-AAAB-2D9CB778713C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F13A5E8-21BD-4FAC-9CBC-DD935BB0BED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{447C774D-20D4-470A-ABC0-4D0CBA5C9366}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{447C774D-20D4-470A-ABC0-4D0CBA5C9366}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,32 +34,124 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Porduct</t>
-  </si>
-  <si>
-    <t>Color</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Donation</t>
-  </si>
-  <si>
-    <t>Saree</t>
-  </si>
-  <si>
-    <t>Blue</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+  <si>
+    <t>TestCaseID</t>
+  </si>
+  <si>
+    <t>TestCaseName</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>TestType</t>
+  </si>
+  <si>
+    <t>ExpectedResult</t>
+  </si>
+  <si>
+    <t>TC001</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>Kurti Navigation</t>
+  </si>
+  <si>
+    <t>Women</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Kurti page should open</t>
+  </si>
+  <si>
+    <t>Pink Tshirt Filter</t>
+  </si>
+  <si>
+    <t>Tshirts</t>
+  </si>
+  <si>
+    <t>Earrings Add To Bag</t>
+  </si>
+  <si>
+    <t>Flats Sorting</t>
+  </si>
+  <si>
+    <t>Size Validation</t>
+  </si>
+  <si>
+    <t>Pincode Validation</t>
+  </si>
+  <si>
+    <t>End To End Flow</t>
+  </si>
+  <si>
+    <t>Earrings</t>
+  </si>
+  <si>
+    <t>Flats</t>
+  </si>
+  <si>
+    <t>Heels</t>
+  </si>
+  <si>
+    <t>Sarees</t>
+  </si>
+  <si>
+    <t>Negative</t>
+  </si>
+  <si>
+    <t>Pink filter should apply</t>
+  </si>
+  <si>
+    <t>Product should add to bag</t>
+  </si>
+  <si>
+    <t>Products should sort high to low</t>
+  </si>
+  <si>
+    <t>Select size validation should display</t>
+  </si>
+  <si>
+    <t>Pincode validation message should display</t>
+  </si>
+  <si>
+    <t>Complete order flow should execute successfully</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -87,8 +179,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,38 +496,152 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C71617A6-438B-4952-A22B-CE7186645599}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="19.6328125" customWidth="1"/>
+    <col min="5" max="5" width="48.36328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
         <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>